<commit_message>
Demo spreadsheets carry the computed values of their formulas. SheetJS wrote the SUM and ratio cells without a result, so viewers and the AI's xlsx reader saw an empty "4분기 합계" column (a test chat said so and added the months up itself).
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/demo/files/groups/재무/2026-4분기-예산.xlsx
+++ b/scripts/demo/files/groups/재무/2026-4분기-예산.xlsx
@@ -443,8 +443,9 @@
       <c r="D2">
         <v>12000000</v>
       </c>
-      <c r="E2" t="e">
+      <c r="E2">
         <f>SUM(B2:D2)</f>
+        <v>47000000</v>
       </c>
       <c r="F2" t="str">
         <v>가을 캠페인 2차 포함</v>
@@ -463,8 +464,9 @@
       <c r="D3">
         <v>104000000</v>
       </c>
-      <c r="E3" t="e">
+      <c r="E3">
         <f>SUM(B3:D3)</f>
+        <v>296000000</v>
       </c>
       <c r="F3" t="str">
         <v>12월 성과급 포함</v>
@@ -483,8 +485,9 @@
       <c r="D4">
         <v>8500000</v>
       </c>
-      <c r="E4" t="e">
+      <c r="E4">
         <f>SUM(B4:D4)</f>
+        <v>25500000</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -503,8 +506,9 @@
       <c r="D5">
         <v>2600000</v>
       </c>
-      <c r="E5" t="e">
+      <c r="E5">
         <f>SUM(B5:D5)</f>
+        <v>7200000</v>
       </c>
       <c r="F5" t="str">
         <v>AI 구독 포함</v>
@@ -523,8 +527,9 @@
       <c r="D6">
         <v>1500000</v>
       </c>
-      <c r="E6" t="e">
+      <c r="E6">
         <f>SUM(B6:D6)</f>
+        <v>6500000</v>
       </c>
       <c r="F6" t="str">
         <v>11월 박람회</v>
@@ -534,17 +539,21 @@
       <c r="A7" t="str">
         <v>합계</v>
       </c>
-      <c r="B7" t="e">
+      <c r="B7">
         <f>SUM(B2:B6)</f>
-      </c>
-      <c r="C7" t="e">
+        <v>128600000</v>
+      </c>
+      <c r="C7">
         <f>SUM(C2:C6)</f>
-      </c>
-      <c r="D7" t="e">
+        <v>125000000</v>
+      </c>
+      <c r="D7">
         <f>SUM(D2:D6)</f>
-      </c>
-      <c r="E7" t="e">
+        <v>128600000</v>
+      </c>
+      <c r="E7">
         <f>SUM(E2:E6)</f>
+        <v>382200000</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -591,8 +600,9 @@
       <c r="C2">
         <v>340000000</v>
       </c>
-      <c r="D2" s="1" t="e">
+      <c r="D2" s="1">
         <f>C2/B2</f>
+        <v>1.0303030303030303</v>
       </c>
     </row>
     <row r="3">
@@ -605,8 +615,9 @@
       <c r="C3">
         <v>310000000</v>
       </c>
-      <c r="D3" s="1" t="e">
+      <c r="D3" s="1">
         <f>C3/B3</f>
+        <v>0.9393939393939394</v>
       </c>
     </row>
     <row r="4">
@@ -619,8 +630,9 @@
       <c r="C4">
         <v>385000000</v>
       </c>
-      <c r="D4" s="1" t="e">
+      <c r="D4" s="1">
         <f>C4/B4</f>
+        <v>1.1</v>
       </c>
     </row>
     <row r="5">

</xml_diff>